<commit_message>
docs: update role requirements matrix
</commit_message>
<xml_diff>
--- a/design_doc/岗位需求分解矩阵.xlsx
+++ b/design_doc/岗位需求分解矩阵.xlsx
@@ -32,12 +32,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="517" uniqueCount="458">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="597" uniqueCount="532">
   <si>
     <t>岗位需求分解矩阵</t>
   </si>
   <si>
-    <t>按业务时间顺序展开：计划确认 → ERP/调拨 → 备料 → 生产报工 → PQC 检验 → 批记录 → 放行。生产组长只上报异常订单，不跟踪、不处理、不扩大化。</t>
+    <t>按业务时间顺序展开：计划确认 → ERP/调拨 → 备料 → 生产报工 → PQC 检验 → 批记录 → 放行。红色为与新流程冲突或需修订的旧内容；绿色为根据新流程新增的岗位/系统需求。</t>
   </si>
   <si>
     <t>职位</t>
@@ -115,36 +115,7 @@
     <t>系统</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FF7F6000"/>
-        <rFont val="宋体"/>
-        <charset val="134"/>
-      </rPr>
-      <t>同步</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FF7F6000"/>
-        <rFont val="Carlito"/>
-        <charset val="134"/>
-      </rPr>
-      <t xml:space="preserve"> ERP </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FF7F6000"/>
-        <rFont val="宋体"/>
-        <charset val="134"/>
-      </rPr>
-      <t>候选数据</t>
-    </r>
+    <t>同步 ERP 候选数据</t>
   </si>
   <si>
     <t>把 ERP 中的生产订单、调拨申请、调拨单、发货数量、物料批次同步到本系统候选池。</t>
@@ -237,109 +208,13 @@
     <t>关联调拨单(注塑件与外采不同)</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="宋体"/>
-        <charset val="134"/>
-      </rPr>
-      <t>把正确的</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Carlito"/>
-        <charset val="134"/>
-      </rPr>
-      <t xml:space="preserve"> ERP </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="宋体"/>
-        <charset val="134"/>
-      </rPr>
-      <t>调拨单关联到对应活跃订单。</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="宋体"/>
-        <charset val="134"/>
-      </rPr>
-      <t>复用现有</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Carlito"/>
-        <charset val="134"/>
-      </rPr>
-      <t xml:space="preserve"> ERP </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="宋体"/>
-        <charset val="134"/>
-      </rPr>
-      <t>库存调拨和</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Carlito"/>
-        <charset val="134"/>
-      </rPr>
-      <t xml:space="preserve"> MES </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="宋体"/>
-        <charset val="134"/>
-      </rPr>
-      <t>调拨单列表作为调拨单查询来源；系统补充活跃订单与调拨单的关联关系，并记录关联人、时间、订单和物料批次追溯信息。</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="宋体"/>
-        <charset val="134"/>
-      </rPr>
-      <t>活跃订单、纸质</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Carlito"/>
-        <charset val="134"/>
-      </rPr>
-      <t xml:space="preserve">/ERP </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="宋体"/>
-        <charset val="134"/>
-      </rPr>
-      <t>调拨单号、物料种类、数量、批次。</t>
-    </r>
+    <t>把正确的 ERP 调拨单关联到对应活跃订单。</t>
+  </si>
+  <si>
+    <t>复用现有 ERP 库存调拨和 MES 调拨单列表作为调拨单查询来源；系统补充活跃订单与调拨单的关联关系，并记录关联人、时间、订单和物料批次追溯信息。</t>
+  </si>
+  <si>
+    <t>活跃订单、纸质/ERP 调拨单号、物料种类、数量、批次。</t>
   </si>
   <si>
     <t>活跃订单与调拨单关联关系。</t>
@@ -348,105 +223,7 @@
     <t>关联后检查该活跃订单能看到调拨单、物料种类、数量和批次；未关联时开工检查阻塞。</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="宋体"/>
-        <charset val="134"/>
-      </rPr>
-      <t>进入工序池班组长工作台的生产组长页签</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Carlito"/>
-        <charset val="134"/>
-      </rPr>
-      <t xml:space="preserve"> → </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="宋体"/>
-        <charset val="134"/>
-      </rPr>
-      <t>选择活跃订单</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Carlito"/>
-        <charset val="134"/>
-      </rPr>
-      <t xml:space="preserve"> → </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="宋体"/>
-        <charset val="134"/>
-      </rPr>
-      <t>从现有</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Carlito"/>
-        <charset val="134"/>
-      </rPr>
-      <t xml:space="preserve"> ERP </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="宋体"/>
-        <charset val="134"/>
-      </rPr>
-      <t>库存调拨或</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Carlito"/>
-        <charset val="134"/>
-      </rPr>
-      <t xml:space="preserve"> MES </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="宋体"/>
-        <charset val="134"/>
-      </rPr>
-      <t>调拨单列表查询调拨单</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Carlito"/>
-        <charset val="134"/>
-      </rPr>
-      <t xml:space="preserve"> → </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="宋体"/>
-        <charset val="134"/>
-      </rPr>
-      <t>核对后关联到活跃订单。</t>
-    </r>
+    <t>进入工序池班组长工作台的生产组长页签 → 选择活跃订单 → 从现有 ERP 库存调拨或 MES 调拨单列表查询调拨单 → 核对后关联到活跃订单。</t>
   </si>
   <si>
     <t>订单开工检查</t>
@@ -485,270 +262,19 @@
     <t>产品、工艺路线、路线版本、工序、检验项目、首检数量、上午巡检比例、下午巡检比例、末检规则、接受标准。</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="宋体"/>
-        <charset val="134"/>
-      </rPr>
-      <t>有效</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Carlito"/>
-        <charset val="134"/>
-      </rPr>
-      <t xml:space="preserve"> QA </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="宋体"/>
-        <charset val="134"/>
-      </rPr>
-      <t>检验规程版本。</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="宋体"/>
-        <charset val="134"/>
-      </rPr>
-      <t>缺首检</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Carlito"/>
-        <charset val="134"/>
-      </rPr>
-      <t>/</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="宋体"/>
-        <charset val="134"/>
-      </rPr>
-      <t>上午巡检</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Carlito"/>
-        <charset val="134"/>
-      </rPr>
-      <t>/</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="宋体"/>
-        <charset val="134"/>
-      </rPr>
-      <t>下午巡检任一规则时，</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Carlito"/>
-        <charset val="134"/>
-      </rPr>
-      <t xml:space="preserve">PQC </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="宋体"/>
-        <charset val="134"/>
-      </rPr>
-      <t>任务生成或提交应阻塞；末检按配置判断。</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="宋体"/>
-        <charset val="134"/>
-      </rPr>
-      <t>进入</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Carlito"/>
-        <charset val="134"/>
-      </rPr>
-      <t xml:space="preserve"> QA </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="宋体"/>
-        <charset val="134"/>
-      </rPr>
-      <t>检验规程配置</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Carlito"/>
-        <charset val="134"/>
-      </rPr>
-      <t xml:space="preserve"> → </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="宋体"/>
-        <charset val="134"/>
-      </rPr>
-      <t>选择产品</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Carlito"/>
-        <charset val="134"/>
-      </rPr>
-      <t>/</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="宋体"/>
-        <charset val="134"/>
-      </rPr>
-      <t>路线</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Carlito"/>
-        <charset val="134"/>
-      </rPr>
-      <t>/</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="宋体"/>
-        <charset val="134"/>
-      </rPr>
-      <t>版本</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Carlito"/>
-        <charset val="134"/>
-      </rPr>
-      <t>/</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="宋体"/>
-        <charset val="134"/>
-      </rPr>
-      <t>工序</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Carlito"/>
-        <charset val="134"/>
-      </rPr>
-      <t xml:space="preserve"> → </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="宋体"/>
-        <charset val="134"/>
-      </rPr>
-      <t>填规则</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Carlito"/>
-        <charset val="134"/>
-      </rPr>
-      <t xml:space="preserve"> → </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="宋体"/>
-        <charset val="134"/>
-      </rPr>
-      <t>发布有效版本。</t>
-    </r>
+    <t>有效 QA 检验规程版本。</t>
+  </si>
+  <si>
+    <t>缺首检/上午巡检/下午巡检任一规则时，PQC 任务生成或提交应阻塞；末检按配置判断。</t>
+  </si>
+  <si>
+    <t>进入 QA 检验规程配置 → 选择产品/路线/版本/工序 → 填规则 → 发布有效版本。</t>
   </si>
   <si>
     <t>生产员工</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FF7F6000"/>
-        <rFont val="宋体"/>
-        <charset val="134"/>
-      </rPr>
-      <t>按</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FF7F6000"/>
-        <rFont val="Carlito"/>
-        <charset val="134"/>
-      </rPr>
-      <t xml:space="preserve"> SOP </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FF7F6000"/>
-        <rFont val="宋体"/>
-        <charset val="134"/>
-      </rPr>
-      <t>生产</t>
-    </r>
+    <t>按 SOP 生产</t>
   </si>
   <si>
     <t>一线员工根据每个产品、每个工序对应的 SOP 进行实际生产。</t>
@@ -769,25 +295,25 @@
     <t>按班组安排和 SOP 生产，完成一段后进入生产填写。</t>
   </si>
   <si>
-    <t>生产报工</t>
-  </si>
-  <si>
-    <t>生产结束后报工，填写自己负责的工序、每个设备、设备参数、完成数量、损耗数量和损耗原因。</t>
-  </si>
-  <si>
-    <t>复用现有生产填写入口记录原始生产事实；员工选择工序、实际员工、设备和设备参数，系统保留现场上下文，订单归属由班组长后续分配到活跃订单时确定。</t>
-  </si>
-  <si>
-    <t>工序、实际员工、设备、设备参数、完成数量、损耗数量、损耗原因、电子签名。</t>
-  </si>
-  <si>
-    <t>原始报工记录。</t>
-  </si>
-  <si>
-    <t>提交一笔报工后，检查原始员工、工序、设备参数、完成数量、损耗信息均保存且不可被组长覆盖。</t>
-  </si>
-  <si>
-    <t>进入生产填写入口 → 选择工序和实际员工 → 填设备、设备参数、完成数量、损耗数量和损耗原因 → 签名提交。</t>
+    <t>生产报工【冲突：新流程要求提交时选择活跃订单】</t>
+  </si>
+  <si>
+    <t>生产结束后报工，填写自己负责的工序、每个设备、设备参数、完成数量、损耗数量和损耗原因。冲突标注：新流程要求一线生产提交时选择活跃订单，并将提交数量默认自动分配到该活跃订单。</t>
+  </si>
+  <si>
+    <t>复用现有生产填写入口记录原始生产事实。冲突标注：原矩阵写订单归属由班组长后续分配确定；新流程要求新增订单分配链路，提交时先选活跃订单并默认分配，同时保留组长后续调整能力。</t>
+  </si>
+  <si>
+    <t>工序、实际员工、设备、设备参数、完成数量、损耗数量、损耗原因、电子签名、活跃订单。</t>
+  </si>
+  <si>
+    <t>原始报工记录、默认活跃订单分配记录、可供组长调整的报工数量池。</t>
+  </si>
+  <si>
+    <t>提交一笔报工时选择活跃订单，检查原始报工事实保存、数量默认分配到该活跃订单，且员工原始数据不可被组长覆盖。</t>
+  </si>
+  <si>
+    <t>进入生产填写入口 → 选择工序和实际员工 → 选择活跃订单 → 填设备、设备参数、完成数量、损耗数量和损耗原因 → 签名提交。</t>
   </si>
   <si>
     <t>PQC 检验员</t>
@@ -898,25 +424,25 @@
     <t>进入工序池班组长工作台的生产组长页签 → 打开报工确认工作台 → 查看明细 → 通过或退回。</t>
   </si>
   <si>
-    <t>分配报工到生产订单</t>
-  </si>
-  <si>
-    <t>把每个工序的报工数量分配给对应活跃生产订单。</t>
-  </si>
-  <si>
-    <t>复用工序池班组长工作台的活跃订单分配能力；系统展示可分配报工、活跃订单、工序应完成数量和剩余数量。生产订单数量使用 ERP 下达后的固定产品数量，工序应完成数量 = 固定生产订单数量 × 工序生产系数，报工分配不改变订单产品数量。</t>
-  </si>
-  <si>
-    <t>已复核报工、活跃订单、工序、ERP 下达后的固定生产订单数量、工序生产系数、已分配数量。</t>
-  </si>
-  <si>
-    <t>报工分配记录和订单工序进度。</t>
-  </si>
-  <si>
-    <t>ERP 下达生产订单数量为 300 时，生产系数 1.0 的工序应完成 300，生产系数 3.0 的工序应完成 900；多次报工分配后订单产品数量仍为 300，只更新工序已完成和剩余数量。</t>
-  </si>
-  <si>
-    <t>进入工序池班组长工作台的生产组长页签 → 报工确认工作台 → 选择 FIFO 建议或手动调整 → 分配到活跃订单 → 提交复核。</t>
+    <t>分配报工到生产订单【冲突/补充：一线提交后已默认分配，组长可重新分配】</t>
+  </si>
+  <si>
+    <t>把每个工序的报工数量分配给对应活跃生产订单。冲突标注：新流程要求一线提交后先自动分配到其选择的活跃订单；生产组长在报工管理列表中仍可把数量重新分配给其他订单。</t>
+  </si>
+  <si>
+    <t>复用工序池班组长工作台的活跃订单分配能力；系统展示可分配报工、默认分配订单、可调整订单、工序应完成数量和剩余数量。提交数量超过活跃订单数量时仍允许提交，超量订单在报工管理列表中红色标识。</t>
+  </si>
+  <si>
+    <t>已复核报工、默认活跃订单、可调整活跃订单、工序、ERP 下达后的固定生产订单数量、工序生产系数、已分配数量。</t>
+  </si>
+  <si>
+    <t>报工分配记录、订单工序进度、超量红色标识、组长调整审计记录。</t>
+  </si>
+  <si>
+    <t>提交数量超过默认活跃订单数量时仍提交成功；生产组长列表对应订单红色标识；组长把部分或全部数量调整到其他订单后，进度和标识重新计算。</t>
+  </si>
+  <si>
+    <t>进入工序池班组长工作台的生产组长页签 → 报工管理列表 → 查看红色超量订单 → 选择 FIFO 建议或手动调整 → 分配到其他活跃订单 → 保存。</t>
   </si>
   <si>
     <t>更新生产订单进度</t>
@@ -1006,49 +532,274 @@
     <t>PQC 组长在工序池班组长工作台确认检验提交后，系统自动汇集；PQC 组长和放行负责人查看过程检验记录状态。</t>
   </si>
   <si>
-    <t>检查批记录完整性</t>
-  </si>
-  <si>
-    <t>当生产订单所有工序批记录表单和对应过程检验记录都填完后，判定订单具备放行条件。</t>
-  </si>
-  <si>
-    <t>复用电子批记录和放行追溯的完整性检查能力；系统围绕活跃订单检查工序进度、批记录表单、PQC 组长确认后的过程检验记录和异常状态。</t>
+    <t>检查批记录完整性【冲突：原矩阵缺少双 100% 完工按钮和生产放行阶段】</t>
+  </si>
+  <si>
+    <t>当生产订单所有工序批记录表单和对应过程检验记录都填完后，判定订单具备放行条件。冲突标注：新流程要求生产进度 100% 且检测进度 100% 后，由生产组长点击完工，再进入生产放行阶段。</t>
+  </si>
+  <si>
+    <t>复用电子批记录和放行追溯的完整性检查能力；需补充生产进度 100%、检测进度 100%、生产组长完工按钮、完工后推送 PQC 负责人生产放行。</t>
   </si>
   <si>
     <t>订单工序进度、批记录表单状态、过程检验记录状态、异常订单状态。</t>
   </si>
   <si>
-    <t>完整性检查结果和放行待办触发条件。</t>
-  </si>
-  <si>
-    <t>缺任一批记录或过程检验记录时不得生成放行待办；全部完成时生成放行待办。</t>
-  </si>
-  <si>
-    <t>进入电子批记录放行追溯 → 查看检查项 → 核对批记录、过程检验记录和异常状态 → 缺项按系统提示回到对应角色补齐。</t>
+    <t>完整性检查结果、双 100% 完工触发条件、生产放行待办触发条件。</t>
+  </si>
+  <si>
+    <t>生产进度或检测进度未到 100% 时不能完工；双 100% 后生产组长点击完工，系统生成 PQC 负责人生产放行待办。</t>
+  </si>
+  <si>
+    <t>进入电子批记录放行追溯或生产组长工作台 → 查看生产进度和检测进度 → 双 100% 后点击完工 → 系统推送生产放行。</t>
   </si>
   <si>
     <t>放行负责人</t>
   </si>
   <si>
-    <t>审核并放行生产订单</t>
-  </si>
-  <si>
-    <t>收到系统推送后，审核完整批记录和过程检验记录，决定放行或退回。</t>
-  </si>
-  <si>
-    <t>复用电子批记录放行追溯页面；系统展示完整批记录、过程检验记录、物料批次、人员签名和异常状态，放行负责人在此完成放行或退回。</t>
-  </si>
-  <si>
-    <t>完整批记录、过程检验记录、物料追溯、电子签名、完整性检查结果。</t>
-  </si>
-  <si>
-    <t>放行结果或退回原因。</t>
-  </si>
-  <si>
-    <t>完整订单应能放行；缺记录或存在阻塞异常时不能放行或必须退回说明原因。</t>
-  </si>
-  <si>
-    <t>进入电子批记录放行追溯 → 打开放行检查项和批记录资料 → 审核过程检验记录、物料批次和签名 → 放行或退回。</t>
+    <t>审核并放行生产订单【冲突：原矩阵放行链路过粗】</t>
+  </si>
+  <si>
+    <t>收到系统推送后，审核完整批记录和过程检验记录，决定放行或退回。冲突标注：新流程将放行拆分为 PQC 生产放行、三份报告上传、管理者代表授权者批记录放行，最后进入可追溯列表。</t>
+  </si>
+  <si>
+    <t>复用电子批记录放行追溯页面；需补充多阶段待办流转：PQC 负责人生产放行后，推送灭菌负责人、来料检负责人、成品检负责人上传报告；三份报告上传结束后推送管理者代表授权者做批记录放行。</t>
+  </si>
+  <si>
+    <t>完整批记录、过程检验记录、物料追溯、电子签名、完整性检查结果、灭菌报告、来料检报告、成品检报告。</t>
+  </si>
+  <si>
+    <t>生产放行结果、三份报告上传状态、批记录放行结果、可追溯列表记录。</t>
+  </si>
+  <si>
+    <t>PQC 放行后必须分别生成三份报告上传待办；三份报告未齐套不能进入批记录放行；批记录放行后订单进入可追溯列表。</t>
+  </si>
+  <si>
+    <t>PQC 负责人完成生产放行 → 三类负责人上传对应报告 → 管理者代表授权者批记录放行 → 系统进入可追溯列表。</t>
+  </si>
+  <si>
+    <t>生产员工 / 系统</t>
+  </si>
+  <si>
+    <t>新增：提交时选择活跃订单并默认分配</t>
+  </si>
+  <si>
+    <t>一线生产提交报工时选择一个活跃订单，提交后数量自动分配到该订单。</t>
+  </si>
+  <si>
+    <t>在生产填写提交链路中增加活跃订单选择和默认分配记录；原始报工事实与订单分配记录分开保存，便于组长后续调整。</t>
+  </si>
+  <si>
+    <t>活跃订单、报工数量、工序、实际员工、设备参数、电子签名。</t>
+  </si>
+  <si>
+    <t>原始报工记录、默认订单分配记录。</t>
+  </si>
+  <si>
+    <t>选择活跃订单提交后，检查该订单获得默认分配数量，原始报工事实仍独立可追溯。</t>
+  </si>
+  <si>
+    <t>生产填写 → 选择活跃订单 → 填数量和设备参数 → 签名提交。</t>
+  </si>
+  <si>
+    <t>新增：超出活跃订单数量仍允许提交</t>
+  </si>
+  <si>
+    <t>一线提交数量超过所选活跃订单数量时，系统不阻止提交。</t>
+  </si>
+  <si>
+    <t>提交保存原始数量；分配层记录超量状态，供生产组长在报工管理列表处理。</t>
+  </si>
+  <si>
+    <t>所选活跃订单、订单数量、本次提交数量。</t>
+  </si>
+  <si>
+    <t>超量报工事实、超量分配状态。</t>
+  </si>
+  <si>
+    <t>本次提交数量大于订单数量时，提交成功且不丢失超出数量。</t>
+  </si>
+  <si>
+    <t>一线照常提交；系统保存并标记超量。</t>
+  </si>
+  <si>
+    <t>新增：报工管理列表红色标识超量订单</t>
+  </si>
+  <si>
+    <t>生产组长看到报工管理列表时，本次提交所选订单若超量，要用红色标识。</t>
+  </si>
+  <si>
+    <t>列表按默认分配订单、订单数量和本次提交数量计算超量标识；红色仅提示异常，不阻断后续调整。</t>
+  </si>
+  <si>
+    <t>报工记录、默认活跃订单、订单数量、提交数量。</t>
+  </si>
+  <si>
+    <t>红色超量订单标识。</t>
+  </si>
+  <si>
+    <t>构造超量提交，生产组长列表中该订单行或标识为红色；非超量不标红。</t>
+  </si>
+  <si>
+    <t>生产组长页签 → 报工管理列表 → 查看红色超量提示。</t>
+  </si>
+  <si>
+    <t>新增：提交后仍可重新分配到其他订单</t>
+  </si>
+  <si>
+    <t>一线提交后，生产组长可以将本次提交数量分配给其他活跃订单。</t>
+  </si>
+  <si>
+    <t>分配界面提供默认订单和其他可选活跃订单；保存调整记录、分配版本和审计原因。</t>
+  </si>
+  <si>
+    <t>报工数量池、默认订单、目标活跃订单、调整数量、调整原因。</t>
+  </si>
+  <si>
+    <t>重新分配记录、订单进度更新、调整审计。</t>
+  </si>
+  <si>
+    <t>把默认订单的一部分数量转给其他订单后，两个订单进度正确更新，原始报工不被覆盖。</t>
+  </si>
+  <si>
+    <t>报工管理列表 → 打开分配 → 调整目标订单和数量 → 保存。</t>
+  </si>
+  <si>
+    <t>生产班组长 / 系统</t>
+  </si>
+  <si>
+    <t>新增：双 100% 后点击完工</t>
+  </si>
+  <si>
+    <t>生产进度达到 100%、检测进度达到 100% 后，生产组长点击完工按钮。</t>
+  </si>
+  <si>
+    <t>系统校验生产进度和检测进度均为 100%；未满足时阻止完工，满足时生成生产放行待办。</t>
+  </si>
+  <si>
+    <t>生产进度、检测进度、活跃订单、生产组长身份。</t>
+  </si>
+  <si>
+    <t>完工状态、生产放行待办。</t>
+  </si>
+  <si>
+    <t>生产或检测任一未达 100% 时完工按钮不可成功；双 100% 时点击成功并进入下一阶段。</t>
+  </si>
+  <si>
+    <t>生产组长工作台 → 查看进度 → 点击完工。</t>
+  </si>
+  <si>
+    <t>PQC 负责人</t>
+  </si>
+  <si>
+    <t>新增：生产放行</t>
+  </si>
+  <si>
+    <t>完工后推送到 PQC 负责人进行生产放行。</t>
+  </si>
+  <si>
+    <t>建立生产放行待办，PQC 负责人审核生产记录、过程检验记录和完整性检查后放行或退回。</t>
+  </si>
+  <si>
+    <t>完工订单、批记录、过程检验记录、生产放行待办。</t>
+  </si>
+  <si>
+    <t>PQC 生产放行结果或退回原因。</t>
+  </si>
+  <si>
+    <t>完工后 PQC 负责人账号能收到待办；放行后进入三份报告上传阶段。</t>
+  </si>
+  <si>
+    <t>PQC 负责人待办 → 查看资料 → 生产放行。</t>
+  </si>
+  <si>
+    <t>灭菌负责人 / 来料检负责人 / 成品检负责人</t>
+  </si>
+  <si>
+    <t>新增：三份报告上传</t>
+  </si>
+  <si>
+    <t>PQC 生产放行后，分别推送灭菌报告、来料检报告、成品检报告上传任务。</t>
+  </si>
+  <si>
+    <t>系统按三类负责人生成独立上传待办；三份报告状态分别跟踪，全部上传完成后才进入批记录放行。</t>
+  </si>
+  <si>
+    <t>PQC 放行结果、三类负责人、灭菌报告、来料检报告、成品检报告。</t>
+  </si>
+  <si>
+    <t>三份报告文件和上传状态。</t>
+  </si>
+  <si>
+    <t>只上传一份或两份报告时不能进入批记录放行；三份全部上传后自动触发下一阶段。</t>
+  </si>
+  <si>
+    <t>对应负责人待办 → 上传对应报告 → 提交。</t>
+  </si>
+  <si>
+    <t>新增：三份报告齐套后推送批记录放行</t>
+  </si>
+  <si>
+    <t>灭菌、来料检、成品检三份报告上传结束后，系统推送管理者代表授权者进行批记录放行。</t>
+  </si>
+  <si>
+    <t>系统监听三份报告齐套状态；齐套后生成批记录放行待办，未齐套时保持等待。</t>
+  </si>
+  <si>
+    <t>三份报告上传状态、放行订单、批记录资料。</t>
+  </si>
+  <si>
+    <t>管理者代表授权者批记录放行待办。</t>
+  </si>
+  <si>
+    <t>任一报告缺失时不推送；三份齐套后只生成一次批记录放行待办。</t>
+  </si>
+  <si>
+    <t>系统自动推送。</t>
+  </si>
+  <si>
+    <t>管理者代表授权者</t>
+  </si>
+  <si>
+    <t>新增：批记录放行</t>
+  </si>
+  <si>
+    <t>管理者代表授权者收到待办后，对批记录进行最终放行。</t>
+  </si>
+  <si>
+    <t>电子批记录放行页面展示完整批记录、过程检验、三份报告和签名审计；授权者放行或退回。</t>
+  </si>
+  <si>
+    <t>完整批记录、过程检验记录、三份报告、电子签名。</t>
+  </si>
+  <si>
+    <t>批记录放行结果或退回原因。</t>
+  </si>
+  <si>
+    <t>资料完整时可放行；资料缺失或退回时不能进入可追溯列表。</t>
+  </si>
+  <si>
+    <t>管理者代表授权者待办 → 审核资料 → 批记录放行。</t>
+  </si>
+  <si>
+    <t>新增：进入可追溯列表</t>
+  </si>
+  <si>
+    <t>批记录放行完成后，订单进入可追溯列表。</t>
+  </si>
+  <si>
+    <t>系统将放行完成的订单、批记录、报告、物料和签名审计汇总到可追溯列表。</t>
+  </si>
+  <si>
+    <t>批记录放行结果、订单、批记录、三份报告、物料批次、签名审计。</t>
+  </si>
+  <si>
+    <t>可追溯列表记录。</t>
+  </si>
+  <si>
+    <t>批记录放行后可在可追溯列表查询到该订单；未放行订单不得出现。</t>
+  </si>
+  <si>
+    <t>可追溯列表 → 按订单查询。</t>
   </si>
   <si>
     <t>岗位衍生需求分解矩阵</t>
@@ -1535,9 +1286,6 @@
   </si>
   <si>
     <t>完整规程草稿、发布人、发布时间。</t>
-  </si>
-  <si>
-    <t>有效 QA 检验规程版本。</t>
   </si>
   <si>
     <t>发布新版本后，确认新任务用新版本；旧检验记录仍显示当时版本。</t>
@@ -2635,7 +2383,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="38">
+  <fonts count="35">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -2680,71 +2428,54 @@
       <charset val="134"/>
     </font>
     <font>
-      <b/>
       <sz val="16"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Carlito"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="10"/>
-      <color rgb="FF1F4E78"/>
-      <name val="Carlito"/>
+      <name val="微软雅黑"/>
       <charset val="134"/>
     </font>
     <font>
       <b/>
-      <sz val="11"/>
+      <sz val="16"/>
       <color rgb="FFFFFFFF"/>
-      <name val="Carlito"/>
+      <name val="微软雅黑"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <color rgb="FFFF0000"/>
+      <name val="微软雅黑"/>
       <charset val="134"/>
     </font>
     <font>
       <b/>
-      <sz val="10"/>
+      <sz val="16"/>
       <color rgb="FF375623"/>
-      <name val="Carlito"/>
+      <name val="微软雅黑"/>
       <charset val="134"/>
     </font>
     <font>
       <b/>
-      <sz val="10"/>
+      <sz val="16"/>
       <color rgb="FF7F6000"/>
-      <name val="宋体"/>
+      <name val="微软雅黑"/>
       <charset val="134"/>
     </font>
     <font>
-      <sz val="10"/>
+      <sz val="16"/>
       <color rgb="FF222222"/>
-      <name val="Carlito"/>
+      <name val="微软雅黑"/>
       <charset val="134"/>
     </font>
     <font>
       <b/>
-      <sz val="10"/>
-      <color rgb="FF7F6000"/>
-      <name val="Carlito"/>
+      <sz val="16"/>
+      <color rgb="FFFF0000"/>
+      <name val="微软雅黑"/>
       <charset val="134"/>
     </font>
     <font>
-      <b/>
-      <sz val="10"/>
-      <color rgb="FFFF0000"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FFFF0000"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
-      <color rgb="FFFF0000"/>
-      <name val="Carlito"/>
+      <sz val="16"/>
+      <color rgb="FF008000"/>
+      <name val="微软雅黑"/>
       <charset val="134"/>
     </font>
     <font>
@@ -2898,12 +2629,6 @@
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FFFF0000"/>
-      <name val="Carlito"/>
-      <charset val="134"/>
-    </font>
   </fonts>
   <fills count="40">
     <fill>
@@ -2932,7 +2657,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFEAF3F8"/>
+        <fgColor rgb="FFFCE4D6"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -3141,7 +2866,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="12">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -3176,6 +2901,21 @@
       </top>
       <bottom style="thin">
         <color rgb="FFD9E2F3"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
       </bottom>
       <diagonal/>
     </border>
@@ -3297,19 +3037,28 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="17" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="15" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="17" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="44" fontId="15" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="17" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="9" fontId="15" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="17" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="41" fontId="15" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="42" fontId="17" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="42" fontId="15" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -3318,127 +3067,118 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="10" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="11" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="10" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="11" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="11" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="12" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="11" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="12" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="30" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="31" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="32" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="33" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="34" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="34" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="33" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="33" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="34" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="34" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="33" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="33" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="34" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="34" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="33" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="33" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="34" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="34" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="33" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="33" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="34" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="34" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="33" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="33" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="34" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="34" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="33" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -3459,44 +3199,44 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="49" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="49" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="49" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="49" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="3" xfId="49" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="49" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="4" xfId="49" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="7" borderId="2" xfId="49" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="8" borderId="2" xfId="49" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="2" xfId="49" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="8" borderId="2" xfId="49" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="2" xfId="49" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="2" xfId="49" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="2" xfId="49" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="50">
@@ -3775,8 +3515,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="RoleRequirementMatrix" displayName="RoleRequirementMatrix" ref="A4:H27" totalsRowShown="0">
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A4:H27" etc:filterBottomFollowUsedRange="0"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="RoleRequirementMatrix" displayName="RoleRequirementMatrix" ref="A4:H37" totalsRowShown="0">
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A4:H37" etc:filterBottomFollowUsedRange="0"/>
   <tableColumns count="8">
     <tableColumn id="1" name="职位"/>
     <tableColumn id="2" name="业务场景/任务"/>
@@ -3986,242 +3726,249 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:H27"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelCol="7"/>
+  <dimension ref="A1:H37"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="22.5" outlineLevelCol="7"/>
   <cols>
-    <col min="1" max="1" width="18" customWidth="1"/>
-    <col min="2" max="2" width="22" customWidth="1"/>
-    <col min="3" max="3" width="36" customWidth="1"/>
-    <col min="4" max="4" width="42" customWidth="1"/>
-    <col min="5" max="5" width="34" customWidth="1"/>
-    <col min="6" max="6" width="32" customWidth="1"/>
-    <col min="7" max="7" width="42" customWidth="1"/>
-    <col min="8" max="8" width="36" customWidth="1"/>
+    <col min="1" max="1" width="20" style="7" customWidth="1"/>
+    <col min="2" max="2" width="30" style="7" customWidth="1"/>
+    <col min="3" max="3" width="48" style="7" customWidth="1"/>
+    <col min="4" max="4" width="62" style="7" customWidth="1"/>
+    <col min="5" max="5" width="40" style="7" customWidth="1"/>
+    <col min="6" max="6" width="38" style="7" customWidth="1"/>
+    <col min="7" max="7" width="48" style="7" customWidth="1"/>
+    <col min="8" max="8" width="44" style="7" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="19.2" customHeight="1" spans="1:8">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" customHeight="1" spans="1:8">
-      <c r="A2" s="8" t="s">
+    <row r="2" ht="60" customHeight="1" spans="1:8">
+      <c r="A2" s="9" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" customHeight="1" spans="1:8">
-      <c r="A4" s="9" t="s">
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
+    </row>
+    <row r="4" ht="15" customHeight="1" spans="1:8">
+      <c r="A4" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="B4" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="C4" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="9" t="s">
+      <c r="D4" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="9" t="s">
+      <c r="E4" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="9" t="s">
+      <c r="F4" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="G4" s="9" t="s">
+      <c r="G4" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="H4" s="9" t="s">
+      <c r="H4" s="10" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="5" ht="36" customHeight="1" spans="1:8">
-      <c r="A5" s="10" t="s">
+    <row r="5" ht="120" customHeight="1" spans="1:8">
+      <c r="A5" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="11" t="s">
+      <c r="B5" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="12" t="s">
+      <c r="C5" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="12" t="s">
+      <c r="D5" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="E5" s="12" t="s">
+      <c r="E5" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="F5" s="12" t="s">
+      <c r="F5" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="G5" s="12" t="s">
+      <c r="G5" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="H5" s="12" t="s">
+      <c r="H5" s="13" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="6" ht="36" customHeight="1" spans="1:8">
-      <c r="A6" s="10" t="s">
+    <row r="6" ht="120" customHeight="1" spans="1:8">
+      <c r="A6" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="B6" s="11" t="s">
+      <c r="B6" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="C6" s="12" t="s">
+      <c r="C6" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="D6" s="12" t="s">
+      <c r="D6" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="E6" s="12" t="s">
+      <c r="E6" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="F6" s="12" t="s">
+      <c r="F6" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="G6" s="12" t="s">
+      <c r="G6" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="H6" s="12" t="s">
+      <c r="H6" s="13" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="7" ht="36" customHeight="1" spans="1:8">
-      <c r="A7" s="10" t="s">
+    <row r="7" ht="120" customHeight="1" spans="1:8">
+      <c r="A7" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="B7" s="11" t="s">
+      <c r="B7" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="C7" s="12" t="s">
+      <c r="C7" s="13" t="s">
         <v>28</v>
       </c>
       <c r="D7" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="E7" s="12" t="s">
+      <c r="E7" s="13" t="s">
         <v>30</v>
       </c>
       <c r="F7" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="G7" s="12" t="s">
+      <c r="G7" s="13" t="s">
         <v>32</v>
       </c>
       <c r="H7" s="13" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="8" ht="24" customHeight="1" spans="1:8">
-      <c r="A8" s="10" t="s">
+    <row r="8" ht="120" customHeight="1" spans="1:8">
+      <c r="A8" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="B8" s="14" t="s">
+      <c r="B8" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="C8" s="12" t="s">
+      <c r="C8" s="13" t="s">
         <v>35</v>
       </c>
       <c r="D8" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="E8" s="12" t="s">
+      <c r="E8" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="F8" s="12" t="s">
+      <c r="F8" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="G8" s="12" t="s">
+      <c r="G8" s="13" t="s">
         <v>39</v>
       </c>
       <c r="H8" s="13" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="9" ht="36" customHeight="1" spans="1:8">
-      <c r="A9" s="10" t="s">
+    <row r="9" ht="120" customHeight="1" spans="1:8">
+      <c r="A9" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="B9" s="14" t="s">
+      <c r="B9" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="C9" s="12" t="s">
+      <c r="C9" s="13" t="s">
         <v>43</v>
       </c>
-      <c r="D9" s="12" t="s">
+      <c r="D9" s="13" t="s">
         <v>44</v>
       </c>
-      <c r="E9" s="12" t="s">
+      <c r="E9" s="13" t="s">
         <v>45</v>
       </c>
-      <c r="F9" s="12" t="s">
+      <c r="F9" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="G9" s="12" t="s">
+      <c r="G9" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="H9" s="12" t="s">
+      <c r="H9" s="13" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="10" ht="24" customHeight="1" spans="1:8">
-      <c r="A10" s="10" t="s">
+    <row r="10" ht="120" customHeight="1" spans="1:8">
+      <c r="A10" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="B10" s="14" t="s">
+      <c r="B10" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="C10" s="12" t="s">
+      <c r="C10" s="13" t="s">
         <v>51</v>
       </c>
       <c r="D10" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="E10" s="12" t="s">
+      <c r="E10" s="13" t="s">
         <v>53</v>
       </c>
-      <c r="F10" s="12" t="s">
+      <c r="F10" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="G10" s="12" t="s">
+      <c r="G10" s="13" t="s">
         <v>55</v>
       </c>
       <c r="H10" s="13" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="11" s="6" customFormat="1" ht="24" customHeight="1" spans="1:8">
-      <c r="A11" s="15" t="s">
+    <row r="11" s="6" customFormat="1" ht="120" customHeight="1" spans="1:8">
+      <c r="A11" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="16" t="s">
+      <c r="B11" s="15" t="s">
         <v>57</v>
       </c>
-      <c r="C11" s="17" t="s">
+      <c r="C11" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="D11" s="18" t="s">
+      <c r="D11" s="16" t="s">
         <v>59</v>
       </c>
-      <c r="E11" s="17" t="s">
+      <c r="E11" s="16" t="s">
         <v>60</v>
       </c>
-      <c r="F11" s="17" t="s">
+      <c r="F11" s="16" t="s">
         <v>61</v>
       </c>
-      <c r="G11" s="17" t="s">
+      <c r="G11" s="16" t="s">
         <v>62</v>
       </c>
-      <c r="H11" s="18" t="s">
+      <c r="H11" s="16" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="12" ht="36" customHeight="1" spans="1:8">
-      <c r="A12" s="10" t="s">
+    <row r="12" ht="120" customHeight="1" spans="1:8">
+      <c r="A12" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="14" t="s">
+      <c r="B12" s="12" t="s">
         <v>64</v>
       </c>
       <c r="C12" s="13" t="s">
@@ -4230,7 +3977,7 @@
       <c r="D12" s="13" t="s">
         <v>66</v>
       </c>
-      <c r="E12" s="12" t="s">
+      <c r="E12" s="13" t="s">
         <v>67</v>
       </c>
       <c r="F12" s="13" t="s">
@@ -4243,245 +3990,245 @@
         <v>70</v>
       </c>
     </row>
-    <row r="13" s="6" customFormat="1" ht="36" customHeight="1" spans="1:8">
-      <c r="A13" s="19" t="s">
+    <row r="13" s="6" customFormat="1" ht="120" customHeight="1" spans="1:8">
+      <c r="A13" s="14" t="s">
         <v>71</v>
       </c>
-      <c r="B13" s="16" t="s">
+      <c r="B13" s="15" t="s">
         <v>72</v>
       </c>
-      <c r="C13" s="17" t="s">
+      <c r="C13" s="16" t="s">
         <v>73</v>
       </c>
-      <c r="D13" s="17" t="s">
+      <c r="D13" s="16" t="s">
         <v>74</v>
       </c>
-      <c r="E13" s="17" t="s">
+      <c r="E13" s="16" t="s">
         <v>75</v>
       </c>
-      <c r="F13" s="17" t="s">
+      <c r="F13" s="16" t="s">
         <v>76</v>
       </c>
-      <c r="G13" s="17" t="s">
+      <c r="G13" s="16" t="s">
         <v>77</v>
       </c>
-      <c r="H13" s="17" t="s">
+      <c r="H13" s="16" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="14" ht="24" customHeight="1" spans="1:8">
-      <c r="A14" s="10" t="s">
+    <row r="14" ht="120" customHeight="1" spans="1:8">
+      <c r="A14" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="B14" s="11" t="s">
+      <c r="B14" s="12" t="s">
         <v>80</v>
       </c>
-      <c r="C14" s="12" t="s">
+      <c r="C14" s="13" t="s">
         <v>81</v>
       </c>
-      <c r="D14" s="12" t="s">
+      <c r="D14" s="13" t="s">
         <v>82</v>
       </c>
-      <c r="E14" s="12" t="s">
+      <c r="E14" s="13" t="s">
         <v>83</v>
       </c>
-      <c r="F14" s="12" t="s">
+      <c r="F14" s="13" t="s">
         <v>84</v>
       </c>
-      <c r="G14" s="12" t="s">
+      <c r="G14" s="13" t="s">
         <v>85</v>
       </c>
-      <c r="H14" s="12" t="s">
+      <c r="H14" s="13" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="15" ht="36" customHeight="1" spans="1:8">
-      <c r="A15" s="10" t="s">
+    <row r="15" ht="120" customHeight="1" spans="1:8">
+      <c r="A15" s="17" t="s">
         <v>79</v>
       </c>
-      <c r="B15" s="14" t="s">
+      <c r="B15" s="17" t="s">
         <v>87</v>
       </c>
-      <c r="C15" s="12" t="s">
+      <c r="C15" s="18" t="s">
         <v>88</v>
       </c>
-      <c r="D15" s="13" t="s">
+      <c r="D15" s="18" t="s">
         <v>89</v>
       </c>
-      <c r="E15" s="12" t="s">
+      <c r="E15" s="18" t="s">
         <v>90</v>
       </c>
-      <c r="F15" s="12" t="s">
+      <c r="F15" s="18" t="s">
         <v>91</v>
       </c>
-      <c r="G15" s="12" t="s">
+      <c r="G15" s="18" t="s">
         <v>92</v>
       </c>
-      <c r="H15" s="13" t="s">
+      <c r="H15" s="18" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="16" ht="24" customHeight="1" spans="1:8">
-      <c r="A16" s="10" t="s">
+    <row r="16" ht="120" customHeight="1" spans="1:8">
+      <c r="A16" s="11" t="s">
         <v>94</v>
       </c>
-      <c r="B16" s="14" t="s">
+      <c r="B16" s="12" t="s">
         <v>95</v>
       </c>
-      <c r="C16" s="12" t="s">
+      <c r="C16" s="13" t="s">
         <v>96</v>
       </c>
       <c r="D16" s="13" t="s">
         <v>97</v>
       </c>
-      <c r="E16" s="12" t="s">
+      <c r="E16" s="13" t="s">
         <v>98</v>
       </c>
-      <c r="F16" s="12" t="s">
+      <c r="F16" s="13" t="s">
         <v>99</v>
       </c>
-      <c r="G16" s="12" t="s">
+      <c r="G16" s="13" t="s">
         <v>100</v>
       </c>
       <c r="H16" s="13" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="17" ht="24" customHeight="1" spans="1:8">
-      <c r="A17" s="10" t="s">
+    <row r="17" ht="120" customHeight="1" spans="1:8">
+      <c r="A17" s="11" t="s">
         <v>94</v>
       </c>
-      <c r="B17" s="14" t="s">
+      <c r="B17" s="12" t="s">
         <v>102</v>
       </c>
-      <c r="C17" s="12" t="s">
+      <c r="C17" s="13" t="s">
         <v>103</v>
       </c>
       <c r="D17" s="13" t="s">
         <v>104</v>
       </c>
-      <c r="E17" s="12" t="s">
+      <c r="E17" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="F17" s="12" t="s">
+      <c r="F17" s="13" t="s">
         <v>106</v>
       </c>
-      <c r="G17" s="12" t="s">
+      <c r="G17" s="13" t="s">
         <v>107</v>
       </c>
       <c r="H17" s="13" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="18" ht="24" customHeight="1" spans="1:8">
-      <c r="A18" s="10" t="s">
+    <row r="18" ht="120" customHeight="1" spans="1:8">
+      <c r="A18" s="11" t="s">
         <v>94</v>
       </c>
-      <c r="B18" s="14" t="s">
+      <c r="B18" s="12" t="s">
         <v>109</v>
       </c>
-      <c r="C18" s="12" t="s">
+      <c r="C18" s="13" t="s">
         <v>110</v>
       </c>
       <c r="D18" s="13" t="s">
         <v>111</v>
       </c>
-      <c r="E18" s="12" t="s">
+      <c r="E18" s="13" t="s">
         <v>112</v>
       </c>
-      <c r="F18" s="12" t="s">
+      <c r="F18" s="13" t="s">
         <v>113</v>
       </c>
-      <c r="G18" s="12" t="s">
+      <c r="G18" s="13" t="s">
         <v>114</v>
       </c>
       <c r="H18" s="13" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="19" ht="36" customHeight="1" spans="1:8">
-      <c r="A19" s="10" t="s">
+    <row r="19" ht="120" customHeight="1" spans="1:8">
+      <c r="A19" s="11" t="s">
         <v>94</v>
       </c>
-      <c r="B19" s="14" t="s">
+      <c r="B19" s="12" t="s">
         <v>116</v>
       </c>
-      <c r="C19" s="12" t="s">
+      <c r="C19" s="13" t="s">
         <v>117</v>
       </c>
       <c r="D19" s="13" t="s">
         <v>118</v>
       </c>
-      <c r="E19" s="12" t="s">
+      <c r="E19" s="13" t="s">
         <v>119</v>
       </c>
-      <c r="F19" s="12" t="s">
+      <c r="F19" s="13" t="s">
         <v>120</v>
       </c>
-      <c r="G19" s="12" t="s">
+      <c r="G19" s="13" t="s">
         <v>121</v>
       </c>
       <c r="H19" s="13" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="20" ht="24" customHeight="1" spans="1:8">
-      <c r="A20" s="10" t="s">
+    <row r="20" ht="120" customHeight="1" spans="1:8">
+      <c r="A20" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="B20" s="11" t="s">
+      <c r="B20" s="12" t="s">
         <v>123</v>
       </c>
-      <c r="C20" s="12" t="s">
+      <c r="C20" s="13" t="s">
         <v>124</v>
       </c>
       <c r="D20" s="13" t="s">
         <v>125</v>
       </c>
-      <c r="E20" s="12" t="s">
+      <c r="E20" s="13" t="s">
         <v>126</v>
       </c>
-      <c r="F20" s="12" t="s">
+      <c r="F20" s="13" t="s">
         <v>127</v>
       </c>
-      <c r="G20" s="12" t="s">
+      <c r="G20" s="13" t="s">
         <v>128</v>
       </c>
       <c r="H20" s="13" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="21" ht="36" customHeight="1" spans="1:8">
-      <c r="A21" s="10" t="s">
+    <row r="21" ht="120" customHeight="1" spans="1:8">
+      <c r="A21" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="B21" s="14" t="s">
+      <c r="B21" s="17" t="s">
         <v>130</v>
       </c>
-      <c r="C21" s="12" t="s">
+      <c r="C21" s="18" t="s">
         <v>131</v>
       </c>
-      <c r="D21" s="13" t="s">
+      <c r="D21" s="18" t="s">
         <v>132</v>
       </c>
-      <c r="E21" s="13" t="s">
+      <c r="E21" s="18" t="s">
         <v>133</v>
       </c>
-      <c r="F21" s="12" t="s">
+      <c r="F21" s="18" t="s">
         <v>134</v>
       </c>
-      <c r="G21" s="13" t="s">
+      <c r="G21" s="18" t="s">
         <v>135</v>
       </c>
-      <c r="H21" s="13" t="s">
+      <c r="H21" s="18" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="22" ht="36" customHeight="1" spans="1:8">
-      <c r="A22" s="10" t="s">
+    <row r="22" ht="120" customHeight="1" spans="1:8">
+      <c r="A22" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="B22" s="14" t="s">
+      <c r="B22" s="12" t="s">
         <v>137</v>
       </c>
       <c r="C22" s="13" t="s">
@@ -4493,144 +4240,404 @@
       <c r="E22" s="13" t="s">
         <v>140</v>
       </c>
-      <c r="F22" s="12" t="s">
+      <c r="F22" s="13" t="s">
         <v>141</v>
       </c>
       <c r="G22" s="13" t="s">
         <v>142</v>
       </c>
-      <c r="H22" s="12" t="s">
+      <c r="H22" s="13" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="23" ht="36" customHeight="1" spans="1:8">
-      <c r="A23" s="10" t="s">
+    <row r="23" ht="120" customHeight="1" spans="1:8">
+      <c r="A23" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="B23" s="14" t="s">
+      <c r="B23" s="12" t="s">
         <v>144</v>
       </c>
-      <c r="C23" s="12" t="s">
+      <c r="C23" s="13" t="s">
         <v>145</v>
       </c>
       <c r="D23" s="13" t="s">
         <v>146</v>
       </c>
-      <c r="E23" s="12" t="s">
+      <c r="E23" s="13" t="s">
         <v>147</v>
       </c>
-      <c r="F23" s="12" t="s">
+      <c r="F23" s="13" t="s">
         <v>148</v>
       </c>
-      <c r="G23" s="12" t="s">
+      <c r="G23" s="13" t="s">
         <v>149</v>
       </c>
       <c r="H23" s="13" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="24" ht="36" customHeight="1" spans="1:8">
-      <c r="A24" s="10" t="s">
+    <row r="24" ht="120" customHeight="1" spans="1:8">
+      <c r="A24" s="11" t="s">
         <v>151</v>
       </c>
-      <c r="B24" s="14" t="s">
+      <c r="B24" s="12" t="s">
         <v>152</v>
       </c>
-      <c r="C24" s="12" t="s">
+      <c r="C24" s="13" t="s">
         <v>153</v>
       </c>
       <c r="D24" s="13" t="s">
         <v>154</v>
       </c>
-      <c r="E24" s="12" t="s">
+      <c r="E24" s="13" t="s">
         <v>155</v>
       </c>
-      <c r="F24" s="12" t="s">
+      <c r="F24" s="13" t="s">
         <v>156</v>
       </c>
-      <c r="G24" s="12" t="s">
+      <c r="G24" s="13" t="s">
         <v>157</v>
       </c>
       <c r="H24" s="13" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="25" ht="36" customHeight="1" spans="1:8">
-      <c r="A25" s="10" t="s">
+    <row r="25" ht="120" customHeight="1" spans="1:8">
+      <c r="A25" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="B25" s="14" t="s">
+      <c r="B25" s="12" t="s">
         <v>159</v>
       </c>
-      <c r="C25" s="12" t="s">
+      <c r="C25" s="13" t="s">
         <v>160</v>
       </c>
       <c r="D25" s="13" t="s">
         <v>161</v>
       </c>
-      <c r="E25" s="12" t="s">
+      <c r="E25" s="13" t="s">
         <v>162</v>
       </c>
-      <c r="F25" s="12" t="s">
+      <c r="F25" s="13" t="s">
         <v>163</v>
       </c>
-      <c r="G25" s="12" t="s">
+      <c r="G25" s="13" t="s">
         <v>164</v>
       </c>
       <c r="H25" s="13" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="26" ht="24" customHeight="1" spans="1:8">
-      <c r="A26" s="10" t="s">
+    <row r="26" ht="120" customHeight="1" spans="1:8">
+      <c r="A26" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="B26" s="14" t="s">
+      <c r="B26" s="17" t="s">
         <v>166</v>
       </c>
-      <c r="C26" s="12" t="s">
+      <c r="C26" s="18" t="s">
         <v>167</v>
       </c>
-      <c r="D26" s="13" t="s">
+      <c r="D26" s="18" t="s">
         <v>168</v>
       </c>
-      <c r="E26" s="12" t="s">
+      <c r="E26" s="18" t="s">
         <v>169</v>
       </c>
-      <c r="F26" s="12" t="s">
+      <c r="F26" s="18" t="s">
         <v>170</v>
       </c>
-      <c r="G26" s="12" t="s">
+      <c r="G26" s="18" t="s">
         <v>171</v>
       </c>
-      <c r="H26" s="13" t="s">
+      <c r="H26" s="18" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="27" ht="24" customHeight="1" spans="1:8">
-      <c r="A27" s="10" t="s">
+    <row r="27" ht="120" customHeight="1" spans="1:8">
+      <c r="A27" s="17" t="s">
         <v>173</v>
       </c>
-      <c r="B27" s="14" t="s">
+      <c r="B27" s="17" t="s">
         <v>174</v>
       </c>
-      <c r="C27" s="12" t="s">
+      <c r="C27" s="18" t="s">
         <v>175</v>
       </c>
-      <c r="D27" s="13" t="s">
+      <c r="D27" s="18" t="s">
         <v>176</v>
       </c>
-      <c r="E27" s="12" t="s">
+      <c r="E27" s="18" t="s">
         <v>177</v>
       </c>
-      <c r="F27" s="12" t="s">
+      <c r="F27" s="18" t="s">
         <v>178</v>
       </c>
-      <c r="G27" s="12" t="s">
+      <c r="G27" s="18" t="s">
         <v>179</v>
       </c>
-      <c r="H27" s="13" t="s">
+      <c r="H27" s="18" t="s">
         <v>180</v>
+      </c>
+    </row>
+    <row r="28" ht="120" customHeight="1" spans="1:8">
+      <c r="A28" s="19" t="s">
+        <v>181</v>
+      </c>
+      <c r="B28" s="19" t="s">
+        <v>182</v>
+      </c>
+      <c r="C28" s="19" t="s">
+        <v>183</v>
+      </c>
+      <c r="D28" s="19" t="s">
+        <v>184</v>
+      </c>
+      <c r="E28" s="19" t="s">
+        <v>185</v>
+      </c>
+      <c r="F28" s="19" t="s">
+        <v>186</v>
+      </c>
+      <c r="G28" s="19" t="s">
+        <v>187</v>
+      </c>
+      <c r="H28" s="19" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="29" ht="120" customHeight="1" spans="1:8">
+      <c r="A29" s="19" t="s">
+        <v>181</v>
+      </c>
+      <c r="B29" s="19" t="s">
+        <v>189</v>
+      </c>
+      <c r="C29" s="19" t="s">
+        <v>190</v>
+      </c>
+      <c r="D29" s="19" t="s">
+        <v>191</v>
+      </c>
+      <c r="E29" s="19" t="s">
+        <v>192</v>
+      </c>
+      <c r="F29" s="19" t="s">
+        <v>193</v>
+      </c>
+      <c r="G29" s="19" t="s">
+        <v>194</v>
+      </c>
+      <c r="H29" s="19" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="30" ht="120" customHeight="1" spans="1:8">
+      <c r="A30" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="B30" s="19" t="s">
+        <v>196</v>
+      </c>
+      <c r="C30" s="19" t="s">
+        <v>197</v>
+      </c>
+      <c r="D30" s="19" t="s">
+        <v>198</v>
+      </c>
+      <c r="E30" s="19" t="s">
+        <v>199</v>
+      </c>
+      <c r="F30" s="19" t="s">
+        <v>200</v>
+      </c>
+      <c r="G30" s="19" t="s">
+        <v>201</v>
+      </c>
+      <c r="H30" s="19" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="31" ht="120" customHeight="1" spans="1:8">
+      <c r="A31" s="19" t="s">
+        <v>18</v>
+      </c>
+      <c r="B31" s="19" t="s">
+        <v>203</v>
+      </c>
+      <c r="C31" s="19" t="s">
+        <v>204</v>
+      </c>
+      <c r="D31" s="19" t="s">
+        <v>205</v>
+      </c>
+      <c r="E31" s="19" t="s">
+        <v>206</v>
+      </c>
+      <c r="F31" s="19" t="s">
+        <v>207</v>
+      </c>
+      <c r="G31" s="19" t="s">
+        <v>208</v>
+      </c>
+      <c r="H31" s="19" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="32" ht="120" customHeight="1" spans="1:8">
+      <c r="A32" s="19" t="s">
+        <v>210</v>
+      </c>
+      <c r="B32" s="19" t="s">
+        <v>211</v>
+      </c>
+      <c r="C32" s="19" t="s">
+        <v>212</v>
+      </c>
+      <c r="D32" s="19" t="s">
+        <v>213</v>
+      </c>
+      <c r="E32" s="19" t="s">
+        <v>214</v>
+      </c>
+      <c r="F32" s="19" t="s">
+        <v>215</v>
+      </c>
+      <c r="G32" s="19" t="s">
+        <v>216</v>
+      </c>
+      <c r="H32" s="19" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="33" ht="120" customHeight="1" spans="1:8">
+      <c r="A33" s="19" t="s">
+        <v>218</v>
+      </c>
+      <c r="B33" s="19" t="s">
+        <v>219</v>
+      </c>
+      <c r="C33" s="19" t="s">
+        <v>220</v>
+      </c>
+      <c r="D33" s="19" t="s">
+        <v>221</v>
+      </c>
+      <c r="E33" s="19" t="s">
+        <v>222</v>
+      </c>
+      <c r="F33" s="19" t="s">
+        <v>223</v>
+      </c>
+      <c r="G33" s="19" t="s">
+        <v>224</v>
+      </c>
+      <c r="H33" s="19" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="34" ht="120" customHeight="1" spans="1:8">
+      <c r="A34" s="19" t="s">
+        <v>226</v>
+      </c>
+      <c r="B34" s="19" t="s">
+        <v>227</v>
+      </c>
+      <c r="C34" s="19" t="s">
+        <v>228</v>
+      </c>
+      <c r="D34" s="19" t="s">
+        <v>229</v>
+      </c>
+      <c r="E34" s="19" t="s">
+        <v>230</v>
+      </c>
+      <c r="F34" s="19" t="s">
+        <v>231</v>
+      </c>
+      <c r="G34" s="19" t="s">
+        <v>232</v>
+      </c>
+      <c r="H34" s="19" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="35" ht="120" customHeight="1" spans="1:8">
+      <c r="A35" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="B35" s="19" t="s">
+        <v>234</v>
+      </c>
+      <c r="C35" s="19" t="s">
+        <v>235</v>
+      </c>
+      <c r="D35" s="19" t="s">
+        <v>236</v>
+      </c>
+      <c r="E35" s="19" t="s">
+        <v>237</v>
+      </c>
+      <c r="F35" s="19" t="s">
+        <v>238</v>
+      </c>
+      <c r="G35" s="19" t="s">
+        <v>239</v>
+      </c>
+      <c r="H35" s="19" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="36" ht="120" customHeight="1" spans="1:8">
+      <c r="A36" s="19" t="s">
+        <v>241</v>
+      </c>
+      <c r="B36" s="19" t="s">
+        <v>242</v>
+      </c>
+      <c r="C36" s="19" t="s">
+        <v>243</v>
+      </c>
+      <c r="D36" s="19" t="s">
+        <v>244</v>
+      </c>
+      <c r="E36" s="19" t="s">
+        <v>245</v>
+      </c>
+      <c r="F36" s="19" t="s">
+        <v>246</v>
+      </c>
+      <c r="G36" s="19" t="s">
+        <v>247</v>
+      </c>
+      <c r="H36" s="19" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="37" ht="120" customHeight="1" spans="1:8">
+      <c r="A37" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="B37" s="19" t="s">
+        <v>249</v>
+      </c>
+      <c r="C37" s="19" t="s">
+        <v>250</v>
+      </c>
+      <c r="D37" s="19" t="s">
+        <v>251</v>
+      </c>
+      <c r="E37" s="19" t="s">
+        <v>252</v>
+      </c>
+      <c r="F37" s="19" t="s">
+        <v>253</v>
+      </c>
+      <c r="G37" s="19" t="s">
+        <v>254</v>
+      </c>
+      <c r="H37" s="19" t="s">
+        <v>255</v>
       </c>
     </row>
   </sheetData>
@@ -4663,7 +4670,7 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:8">
       <c r="A1" s="2" t="s">
-        <v>181</v>
+        <v>256</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -4675,7 +4682,7 @@
     </row>
     <row r="2" ht="34" customHeight="1" spans="1:8">
       <c r="A2" s="3" t="s">
-        <v>182</v>
+        <v>257</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -4691,7 +4698,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>183</v>
+        <v>258</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>4</v>
@@ -4709,7 +4716,7 @@
         <v>8</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>184</v>
+        <v>259</v>
       </c>
     </row>
     <row r="5" ht="66" customHeight="1" spans="1:8">
@@ -4717,25 +4724,25 @@
         <v>18</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>185</v>
+        <v>260</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>186</v>
+        <v>261</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>187</v>
+        <v>262</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>188</v>
+        <v>263</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>189</v>
+        <v>264</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>190</v>
+        <v>265</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>191</v>
+        <v>266</v>
       </c>
     </row>
     <row r="6" ht="66" customHeight="1" spans="1:8">
@@ -4743,25 +4750,25 @@
         <v>18</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>192</v>
+        <v>267</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>193</v>
+        <v>268</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>194</v>
+        <v>269</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>195</v>
+        <v>270</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>196</v>
+        <v>271</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>197</v>
+        <v>272</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>198</v>
+        <v>273</v>
       </c>
     </row>
     <row r="7" ht="66" customHeight="1" spans="1:8">
@@ -4769,25 +4776,25 @@
         <v>18</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>199</v>
+        <v>274</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>200</v>
+        <v>275</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>201</v>
+        <v>276</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>202</v>
+        <v>277</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>203</v>
+        <v>278</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>204</v>
+        <v>279</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>205</v>
+        <v>280</v>
       </c>
     </row>
     <row r="8" ht="66" customHeight="1" spans="1:8">
@@ -4795,25 +4802,25 @@
         <v>18</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>206</v>
+        <v>281</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>207</v>
+        <v>282</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>208</v>
+        <v>283</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>209</v>
+        <v>284</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>210</v>
+        <v>285</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>211</v>
+        <v>286</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>212</v>
+        <v>287</v>
       </c>
     </row>
     <row r="9" ht="66" customHeight="1" spans="1:8">
@@ -4821,25 +4828,25 @@
         <v>18</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>213</v>
+        <v>288</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>214</v>
+        <v>289</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>215</v>
+        <v>290</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>216</v>
+        <v>291</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>217</v>
+        <v>292</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>218</v>
+        <v>293</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>219</v>
+        <v>294</v>
       </c>
     </row>
     <row r="10" ht="66" customHeight="1" spans="1:8">
@@ -4847,25 +4854,25 @@
         <v>18</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>220</v>
+        <v>295</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>221</v>
+        <v>296</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>222</v>
+        <v>297</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>223</v>
+        <v>298</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>224</v>
+        <v>299</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>225</v>
+        <v>300</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>226</v>
+        <v>301</v>
       </c>
     </row>
     <row r="11" ht="66" customHeight="1" spans="1:8">
@@ -4873,25 +4880,25 @@
         <v>18</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>227</v>
+        <v>302</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>228</v>
+        <v>303</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>229</v>
+        <v>304</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>230</v>
+        <v>305</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>231</v>
+        <v>306</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>232</v>
+        <v>307</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>233</v>
+        <v>308</v>
       </c>
     </row>
     <row r="12" ht="66" customHeight="1" spans="1:8">
@@ -4899,25 +4906,25 @@
         <v>18</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>234</v>
+        <v>309</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>235</v>
+        <v>310</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>236</v>
+        <v>311</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>237</v>
+        <v>312</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>238</v>
+        <v>313</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>239</v>
+        <v>314</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>240</v>
+        <v>315</v>
       </c>
     </row>
     <row r="13" ht="66" customHeight="1" spans="1:8">
@@ -4925,25 +4932,25 @@
         <v>18</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>241</v>
+        <v>316</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>242</v>
+        <v>317</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>243</v>
+        <v>318</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>244</v>
+        <v>319</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>245</v>
+        <v>320</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>246</v>
+        <v>321</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>247</v>
+        <v>322</v>
       </c>
     </row>
     <row r="14" ht="66" customHeight="1" spans="1:8">
@@ -4951,25 +4958,25 @@
         <v>18</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>248</v>
+        <v>323</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>249</v>
+        <v>324</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>250</v>
+        <v>325</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>251</v>
+        <v>326</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>252</v>
+        <v>327</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>253</v>
+        <v>328</v>
       </c>
       <c r="H14" s="5" t="s">
-        <v>254</v>
+        <v>329</v>
       </c>
     </row>
     <row r="15" ht="66" customHeight="1" spans="1:8">
@@ -4977,25 +4984,25 @@
         <v>18</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>255</v>
+        <v>330</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>256</v>
+        <v>331</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>257</v>
+        <v>332</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>258</v>
+        <v>333</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>259</v>
+        <v>334</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>260</v>
+        <v>335</v>
       </c>
       <c r="H15" s="5" t="s">
-        <v>261</v>
+        <v>336</v>
       </c>
     </row>
     <row r="16" ht="66" customHeight="1" spans="1:8">
@@ -5003,25 +5010,25 @@
         <v>18</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>262</v>
+        <v>337</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>263</v>
+        <v>338</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>264</v>
+        <v>339</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>265</v>
+        <v>340</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>266</v>
+        <v>341</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>267</v>
+        <v>342</v>
       </c>
       <c r="H16" s="5" t="s">
-        <v>268</v>
+        <v>343</v>
       </c>
     </row>
     <row r="17" ht="66" customHeight="1" spans="1:8">
@@ -5029,25 +5036,25 @@
         <v>18</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>269</v>
+        <v>344</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>270</v>
+        <v>345</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>271</v>
+        <v>346</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>272</v>
+        <v>347</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>273</v>
+        <v>348</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>274</v>
+        <v>349</v>
       </c>
       <c r="H17" s="5" t="s">
-        <v>275</v>
+        <v>350</v>
       </c>
     </row>
     <row r="18" ht="66" customHeight="1" spans="1:8">
@@ -5055,25 +5062,25 @@
         <v>18</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>276</v>
+        <v>351</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>277</v>
+        <v>352</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>278</v>
+        <v>353</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>279</v>
+        <v>354</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>280</v>
+        <v>355</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>281</v>
+        <v>356</v>
       </c>
       <c r="H18" s="5" t="s">
-        <v>282</v>
+        <v>357</v>
       </c>
     </row>
     <row r="19" ht="66" customHeight="1" spans="1:8">
@@ -5081,25 +5088,25 @@
         <v>71</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>283</v>
+        <v>358</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>284</v>
+        <v>359</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>285</v>
+        <v>360</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>286</v>
+        <v>361</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>287</v>
+        <v>362</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>288</v>
+        <v>363</v>
       </c>
       <c r="H19" s="5" t="s">
-        <v>289</v>
+        <v>364</v>
       </c>
     </row>
     <row r="20" ht="66" customHeight="1" spans="1:8">
@@ -5107,25 +5114,25 @@
         <v>71</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>290</v>
+        <v>365</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>291</v>
+        <v>366</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>292</v>
+        <v>367</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>293</v>
+        <v>368</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>294</v>
+        <v>369</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>295</v>
+        <v>370</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>296</v>
+        <v>371</v>
       </c>
     </row>
     <row r="21" ht="66" customHeight="1" spans="1:8">
@@ -5133,25 +5140,25 @@
         <v>71</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>297</v>
+        <v>372</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>298</v>
+        <v>373</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>299</v>
+        <v>374</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>300</v>
+        <v>375</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>301</v>
+        <v>376</v>
       </c>
       <c r="G21" s="5" t="s">
-        <v>302</v>
+        <v>377</v>
       </c>
       <c r="H21" s="5" t="s">
-        <v>303</v>
+        <v>378</v>
       </c>
     </row>
     <row r="22" ht="66" customHeight="1" spans="1:8">
@@ -5159,25 +5166,25 @@
         <v>71</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>304</v>
+        <v>379</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>305</v>
+        <v>380</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>306</v>
+        <v>381</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>307</v>
+        <v>382</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>308</v>
+        <v>383</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>309</v>
+        <v>384</v>
       </c>
       <c r="H22" s="5" t="s">
-        <v>310</v>
+        <v>385</v>
       </c>
     </row>
     <row r="23" ht="66" customHeight="1" spans="1:8">
@@ -5185,25 +5192,25 @@
         <v>71</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>311</v>
+        <v>386</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>312</v>
+        <v>387</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>313</v>
+        <v>388</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>314</v>
+        <v>389</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>315</v>
+        <v>390</v>
       </c>
       <c r="G23" s="5" t="s">
-        <v>316</v>
+        <v>391</v>
       </c>
       <c r="H23" s="5" t="s">
-        <v>317</v>
+        <v>392</v>
       </c>
     </row>
     <row r="24" ht="66" customHeight="1" spans="1:8">
@@ -5211,25 +5218,25 @@
         <v>71</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>318</v>
+        <v>393</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>319</v>
+        <v>394</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>320</v>
+        <v>395</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>321</v>
+        <v>396</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>322</v>
+        <v>397</v>
       </c>
       <c r="G24" s="5" t="s">
-        <v>323</v>
+        <v>398</v>
       </c>
       <c r="H24" s="5" t="s">
-        <v>324</v>
+        <v>399</v>
       </c>
     </row>
     <row r="25" ht="66" customHeight="1" spans="1:8">
@@ -5237,25 +5244,25 @@
         <v>71</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>325</v>
+        <v>400</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>326</v>
+        <v>401</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>327</v>
+        <v>402</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>328</v>
+        <v>403</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>329</v>
+        <v>404</v>
       </c>
       <c r="G25" s="5" t="s">
-        <v>330</v>
+        <v>405</v>
       </c>
       <c r="H25" s="5" t="s">
-        <v>331</v>
+        <v>406</v>
       </c>
     </row>
     <row r="26" ht="66" customHeight="1" spans="1:8">
@@ -5263,25 +5270,25 @@
         <v>71</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>332</v>
+        <v>407</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>333</v>
+        <v>408</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>334</v>
+        <v>409</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>335</v>
+        <v>410</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>336</v>
+        <v>411</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>337</v>
+        <v>412</v>
       </c>
       <c r="H26" s="5" t="s">
-        <v>338</v>
+        <v>413</v>
       </c>
     </row>
     <row r="27" ht="66" customHeight="1" spans="1:8">
@@ -5289,25 +5296,25 @@
         <v>71</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>339</v>
+        <v>414</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>340</v>
+        <v>415</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>341</v>
+        <v>416</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>342</v>
+        <v>417</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>343</v>
+        <v>76</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>344</v>
+        <v>418</v>
       </c>
       <c r="H27" s="5" t="s">
-        <v>345</v>
+        <v>419</v>
       </c>
     </row>
     <row r="28" ht="66" customHeight="1" spans="1:8">
@@ -5315,25 +5322,25 @@
         <v>94</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>346</v>
+        <v>420</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>347</v>
+        <v>421</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>348</v>
+        <v>422</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>349</v>
+        <v>423</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>350</v>
+        <v>424</v>
       </c>
       <c r="G28" s="5" t="s">
-        <v>351</v>
+        <v>425</v>
       </c>
       <c r="H28" s="5" t="s">
-        <v>352</v>
+        <v>426</v>
       </c>
     </row>
     <row r="29" ht="66" customHeight="1" spans="1:8">
@@ -5341,25 +5348,25 @@
         <v>94</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>353</v>
+        <v>427</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>354</v>
+        <v>428</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>355</v>
+        <v>429</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>356</v>
+        <v>430</v>
       </c>
       <c r="F29" s="5" t="s">
-        <v>357</v>
+        <v>431</v>
       </c>
       <c r="G29" s="5" t="s">
-        <v>358</v>
+        <v>432</v>
       </c>
       <c r="H29" s="5" t="s">
-        <v>359</v>
+        <v>433</v>
       </c>
     </row>
     <row r="30" ht="66" customHeight="1" spans="1:8">
@@ -5367,25 +5374,25 @@
         <v>94</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>360</v>
+        <v>434</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>361</v>
+        <v>435</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>362</v>
+        <v>436</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>363</v>
+        <v>437</v>
       </c>
       <c r="F30" s="5" t="s">
-        <v>364</v>
+        <v>438</v>
       </c>
       <c r="G30" s="5" t="s">
-        <v>365</v>
+        <v>439</v>
       </c>
       <c r="H30" s="5" t="s">
-        <v>366</v>
+        <v>440</v>
       </c>
     </row>
     <row r="31" ht="66" customHeight="1" spans="1:8">
@@ -5393,25 +5400,25 @@
         <v>94</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>367</v>
+        <v>441</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>368</v>
+        <v>442</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>369</v>
+        <v>443</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>370</v>
+        <v>444</v>
       </c>
       <c r="F31" s="5" t="s">
-        <v>371</v>
+        <v>445</v>
       </c>
       <c r="G31" s="5" t="s">
-        <v>372</v>
+        <v>446</v>
       </c>
       <c r="H31" s="5" t="s">
-        <v>373</v>
+        <v>447</v>
       </c>
     </row>
     <row r="32" ht="66" customHeight="1" spans="1:8">
@@ -5419,25 +5426,25 @@
         <v>94</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>374</v>
+        <v>448</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>375</v>
+        <v>449</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>376</v>
+        <v>450</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>377</v>
+        <v>451</v>
       </c>
       <c r="F32" s="5" t="s">
-        <v>378</v>
+        <v>452</v>
       </c>
       <c r="G32" s="5" t="s">
-        <v>379</v>
+        <v>453</v>
       </c>
       <c r="H32" s="5" t="s">
-        <v>380</v>
+        <v>454</v>
       </c>
     </row>
     <row r="33" ht="66" customHeight="1" spans="1:8">
@@ -5445,25 +5452,25 @@
         <v>94</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>381</v>
+        <v>455</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>382</v>
+        <v>456</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>383</v>
+        <v>457</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>384</v>
+        <v>458</v>
       </c>
       <c r="F33" s="5" t="s">
-        <v>385</v>
+        <v>459</v>
       </c>
       <c r="G33" s="5" t="s">
-        <v>386</v>
+        <v>460</v>
       </c>
       <c r="H33" s="5" t="s">
-        <v>387</v>
+        <v>461</v>
       </c>
     </row>
     <row r="34" ht="66" customHeight="1" spans="1:8">
@@ -5471,25 +5478,25 @@
         <v>94</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>388</v>
+        <v>462</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>389</v>
+        <v>463</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>390</v>
+        <v>464</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>391</v>
+        <v>465</v>
       </c>
       <c r="F34" s="5" t="s">
-        <v>392</v>
+        <v>466</v>
       </c>
       <c r="G34" s="5" t="s">
-        <v>393</v>
+        <v>467</v>
       </c>
       <c r="H34" s="5" t="s">
-        <v>394</v>
+        <v>468</v>
       </c>
     </row>
     <row r="35" ht="66" customHeight="1" spans="1:8">
@@ -5497,25 +5504,25 @@
         <v>94</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>395</v>
+        <v>469</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>396</v>
+        <v>470</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>397</v>
+        <v>471</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>398</v>
+        <v>472</v>
       </c>
       <c r="F35" s="5" t="s">
-        <v>399</v>
+        <v>473</v>
       </c>
       <c r="G35" s="5" t="s">
-        <v>400</v>
+        <v>474</v>
       </c>
       <c r="H35" s="5" t="s">
-        <v>401</v>
+        <v>475</v>
       </c>
     </row>
     <row r="36" ht="66" customHeight="1" spans="1:8">
@@ -5523,25 +5530,25 @@
         <v>151</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>402</v>
+        <v>476</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>403</v>
+        <v>477</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>404</v>
+        <v>478</v>
       </c>
       <c r="E36" s="5" t="s">
-        <v>405</v>
+        <v>479</v>
       </c>
       <c r="F36" s="5" t="s">
-        <v>406</v>
+        <v>480</v>
       </c>
       <c r="G36" s="5" t="s">
-        <v>407</v>
+        <v>481</v>
       </c>
       <c r="H36" s="5" t="s">
-        <v>408</v>
+        <v>482</v>
       </c>
     </row>
     <row r="37" ht="66" customHeight="1" spans="1:8">
@@ -5549,25 +5556,25 @@
         <v>151</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>409</v>
+        <v>483</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>410</v>
+        <v>484</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>411</v>
+        <v>485</v>
       </c>
       <c r="E37" s="5" t="s">
-        <v>412</v>
+        <v>486</v>
       </c>
       <c r="F37" s="5" t="s">
-        <v>413</v>
+        <v>487</v>
       </c>
       <c r="G37" s="5" t="s">
-        <v>414</v>
+        <v>488</v>
       </c>
       <c r="H37" s="5" t="s">
-        <v>415</v>
+        <v>489</v>
       </c>
     </row>
     <row r="38" ht="66" customHeight="1" spans="1:8">
@@ -5575,25 +5582,25 @@
         <v>151</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>416</v>
+        <v>490</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>417</v>
+        <v>491</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>418</v>
+        <v>492</v>
       </c>
       <c r="E38" s="5" t="s">
-        <v>419</v>
+        <v>493</v>
       </c>
       <c r="F38" s="5" t="s">
         <v>156</v>
       </c>
       <c r="G38" s="5" t="s">
-        <v>420</v>
+        <v>494</v>
       </c>
       <c r="H38" s="5" t="s">
-        <v>421</v>
+        <v>495</v>
       </c>
     </row>
     <row r="39" ht="66" customHeight="1" spans="1:8">
@@ -5601,25 +5608,25 @@
         <v>151</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>422</v>
+        <v>496</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>423</v>
+        <v>497</v>
       </c>
       <c r="D39" s="5" t="s">
-        <v>424</v>
+        <v>498</v>
       </c>
       <c r="E39" s="5" t="s">
-        <v>425</v>
+        <v>499</v>
       </c>
       <c r="F39" s="5" t="s">
-        <v>426</v>
+        <v>500</v>
       </c>
       <c r="G39" s="5" t="s">
-        <v>427</v>
+        <v>501</v>
       </c>
       <c r="H39" s="5" t="s">
-        <v>428</v>
+        <v>502</v>
       </c>
     </row>
     <row r="40" ht="66" customHeight="1" spans="1:8">
@@ -5627,25 +5634,25 @@
         <v>151</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>429</v>
+        <v>503</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>430</v>
+        <v>504</v>
       </c>
       <c r="D40" s="5" t="s">
-        <v>431</v>
+        <v>505</v>
       </c>
       <c r="E40" s="5" t="s">
-        <v>432</v>
+        <v>506</v>
       </c>
       <c r="F40" s="5" t="s">
-        <v>433</v>
+        <v>507</v>
       </c>
       <c r="G40" s="5" t="s">
-        <v>434</v>
+        <v>508</v>
       </c>
       <c r="H40" s="5" t="s">
-        <v>435</v>
+        <v>509</v>
       </c>
     </row>
     <row r="41" ht="66" customHeight="1" spans="1:8">
@@ -5653,25 +5660,25 @@
         <v>151</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>436</v>
+        <v>510</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>437</v>
+        <v>511</v>
       </c>
       <c r="D41" s="5" t="s">
-        <v>438</v>
+        <v>512</v>
       </c>
       <c r="E41" s="5" t="s">
-        <v>439</v>
+        <v>513</v>
       </c>
       <c r="F41" s="5" t="s">
-        <v>440</v>
+        <v>514</v>
       </c>
       <c r="G41" s="5" t="s">
-        <v>441</v>
+        <v>515</v>
       </c>
       <c r="H41" s="5" t="s">
-        <v>442</v>
+        <v>516</v>
       </c>
     </row>
     <row r="42" ht="66" customHeight="1" spans="1:8">
@@ -5679,25 +5686,25 @@
         <v>151</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>443</v>
+        <v>517</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>444</v>
+        <v>518</v>
       </c>
       <c r="D42" s="5" t="s">
-        <v>445</v>
+        <v>519</v>
       </c>
       <c r="E42" s="5" t="s">
-        <v>446</v>
+        <v>520</v>
       </c>
       <c r="F42" s="5" t="s">
-        <v>447</v>
+        <v>521</v>
       </c>
       <c r="G42" s="5" t="s">
-        <v>448</v>
+        <v>522</v>
       </c>
       <c r="H42" s="5" t="s">
-        <v>449</v>
+        <v>523</v>
       </c>
     </row>
     <row r="43" ht="66" customHeight="1" spans="1:8">
@@ -5705,25 +5712,25 @@
         <v>26</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>450</v>
+        <v>524</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>451</v>
+        <v>525</v>
       </c>
       <c r="D43" s="5" t="s">
-        <v>452</v>
+        <v>526</v>
       </c>
       <c r="E43" s="5" t="s">
-        <v>453</v>
+        <v>527</v>
       </c>
       <c r="F43" s="5" t="s">
-        <v>454</v>
+        <v>528</v>
       </c>
       <c r="G43" s="5" t="s">
-        <v>455</v>
+        <v>529</v>
       </c>
       <c r="H43" s="5" t="s">
-        <v>456</v>
+        <v>530</v>
       </c>
     </row>
   </sheetData>
@@ -5748,7 +5755,7 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="1" t="s">
-        <v>457</v>
+        <v>531</v>
       </c>
     </row>
   </sheetData>

</xml_diff>